<commit_message>
feat(01_ERS): RNF de IA (equidad, monitoreo, supervision, riesgo), matriz obligacion legal y vinculo con matriz de trazabilidad
</commit_message>
<xml_diff>
--- a/04_Trazabilidad/Matriz_Trazabilidad_v2.xlsx
+++ b/04_Trazabilidad/Matriz_Trazabilidad_v2.xlsx
@@ -656,12 +656,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Elicitación convencional</t>
+          <t>Res. AGROCALIDAD 183</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Art. 3</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1338,12 +1338,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Elicitación convencional</t>
+          <t>Res. AGROCALIDAD 183</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Art. 36</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1586,12 +1586,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Elicitación convencional</t>
+          <t>Res. AGROCALIDAD 183</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Art. 38 / Art. 18(g) Res.183</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1648,12 +1648,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Elicitación convencional</t>
+          <t>Res. AGROCALIDAD 183</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Art. 27, 29</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Art. 8</t>
+          <t>Art. 4, 8, 10(d), 12(5), 12(8), 34-35 (C1, C2, C3, C5, C12)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Art. 13-19</t>
+          <t>Art. 10(i), 13-19, 33, 36, 43, 46 (C4, C7, C8, C9, C10)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -3880,12 +3880,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Elicitación convencional</t>
+          <t>Res. AGROCALIDAD 183</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Art. 3</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(01_ERS): flujo principal/alternativos por RF, casos de prueba y vinculo en matriz de trazabilidad
</commit_message>
<xml_diff>
--- a/04_Trazabilidad/Matriz_Trazabilidad_v2.xlsx
+++ b/04_Trazabilidad/Matriz_Trazabilidad_v2.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:M61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -528,6 +528,11 @@
           <t>ID-Maqueta</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>ID-Caso-Prueba</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -590,6 +595,11 @@
           <t>MU-02</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>CP-RF-01</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -652,6 +662,11 @@
           <t>MU-02</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>CP-RF-02</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -714,6 +729,11 @@
           <t>MU-03</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>CP-RF-03</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -776,6 +796,11 @@
           <t>MU-04</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>CP-RF-04</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -838,6 +863,11 @@
           <t>MU-08</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>CP-RF-05</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -900,6 +930,11 @@
           <t>MU-08</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>CP-RF-06</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -962,6 +997,11 @@
           <t>MU-05</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>CP-RF-07</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1024,6 +1064,11 @@
           <t>MU-05</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>CP-RF-08</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1086,6 +1131,11 @@
           <t>MU-06</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>CP-RF-09</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1148,6 +1198,11 @@
           <t>MU-06</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>CP-RF-10</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1210,6 +1265,11 @@
           <t>MU-07</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>CP-RF-11</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1272,6 +1332,11 @@
           <t>MU-07</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>CP-RF-12</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1334,6 +1399,11 @@
           <t>MU-04</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>CP-RF-13</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1396,6 +1466,11 @@
           <t>MU-04</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>CP-RF-14</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1458,6 +1533,11 @@
           <t>MU-04</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>CP-RF-15</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1520,6 +1600,11 @@
           <t>MU-02</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>CP-RF-16</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1582,6 +1667,11 @@
           <t>MU-09</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>CP-RF-17</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1644,6 +1734,11 @@
           <t>MU-09</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>CP-RF-18</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1706,6 +1801,11 @@
           <t>MU-08</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>CP-RF-19</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1768,6 +1868,11 @@
           <t>MU-01</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>CP-RF-20</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1830,6 +1935,11 @@
           <t>MU-09</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>CP-RF-21</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1892,6 +2002,11 @@
           <t>MU-01</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>CP-RF-22</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1954,6 +2069,11 @@
           <t>MU-01</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>CP-RF-23</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2016,6 +2136,11 @@
           <t>MU-09</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>CP-RF-24</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2078,6 +2203,11 @@
           <t>MU-09</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>CP-RF-25</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2140,6 +2270,11 @@
           <t>MU-08</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>CP-RF-26</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2202,6 +2337,11 @@
           <t>MU-07</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>CP-RF-27</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2264,6 +2404,11 @@
           <t>MU-07</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>CP-RF-28</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2326,6 +2471,11 @@
           <t>MU-02</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>CP-RF-29</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2388,6 +2538,11 @@
           <t>MU-05</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>CP-RF-30</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2450,6 +2605,11 @@
           <t>MU-06</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>CP-RF-31</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2512,6 +2672,11 @@
           <t>N/A (no se implementará)</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>N/A (Won't have)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2574,6 +2739,11 @@
           <t>MU-06</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>CP-RF-33</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2636,6 +2806,11 @@
           <t>MU-02</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>CP-RF-34</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2698,6 +2873,11 @@
           <t>MU-02</t>
         </is>
       </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>CP-RF-35</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2760,6 +2940,11 @@
           <t>MU-09</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>CP-RF-36</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2822,6 +3007,11 @@
           <t>MU-09</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>CP-RF-37</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2884,6 +3074,11 @@
           <t>MU-09</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>CP-RF-38</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2946,6 +3141,11 @@
           <t>MU-09</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>CP-RF-39</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3008,6 +3208,11 @@
           <t>Transversal (todos los MU)</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>CP-RNF-01</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3070,6 +3275,11 @@
           <t>Transversal (todos los MU)</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>CP-RNF-02</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3132,6 +3342,11 @@
           <t>Transversal (todos los MU)</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>CP-RNF-03</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3194,6 +3409,11 @@
           <t>N/A (no visual)</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>CP-RNF-04</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3256,6 +3476,11 @@
           <t>N/A (no visual)</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>CP-RNF-05</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3318,6 +3543,11 @@
           <t>N/A (no visual)</t>
         </is>
       </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>CP-RNF-06</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3380,6 +3610,11 @@
           <t>N/A (no visual)</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>CP-RNF-07</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3442,6 +3677,11 @@
           <t>N/A (no visual)</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>CP-RNF-08</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3504,6 +3744,11 @@
           <t>N/A (no visual)</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>CP-RNF-09</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3566,6 +3811,11 @@
           <t>N/A (no visual)</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>CP-RNF-10</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3628,6 +3878,11 @@
           <t>N/A (no visual)</t>
         </is>
       </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>CP-RNF-11</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3690,6 +3945,11 @@
           <t>N/A (no visual)</t>
         </is>
       </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>CP-RNF-12</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3752,6 +4012,11 @@
           <t>Transversal (todos los MU)</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>CP-RNF-13</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3814,6 +4079,11 @@
           <t>N/A (no visual)</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>CP-RNF-14</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3876,6 +4146,11 @@
           <t>N/A (no visual)</t>
         </is>
       </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>CP-RNF-15</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3938,6 +4213,11 @@
           <t>MU-06</t>
         </is>
       </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>CP-RF-03</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4000,6 +4280,11 @@
           <t>MU-08</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>CP-RF-01</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4062,6 +4347,11 @@
           <t>MU-08</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>CP-RF-04</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4124,6 +4414,11 @@
           <t>MU-08</t>
         </is>
       </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>CP-RF-07</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4186,6 +4481,11 @@
           <t>MU-05</t>
         </is>
       </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>CP-RF-11</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4246,6 +4546,11 @@
       <c r="L61" s="2" t="inlineStr">
         <is>
           <t>MU-08</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>CP-RF-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: agrega RNF-16 a RNF-21 a matriz de trazabilidad, normaliza comillas en bitacora_sesiones.csv y actualiza checksums
</commit_message>
<xml_diff>
--- a/04_Trazabilidad/Matriz_Trazabilidad_v2.xlsx
+++ b/04_Trazabilidad/Matriz_Trazabilidad_v2.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:M67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4554,6 +4554,408 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Especificación del equipo</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Desempeño de detección/predicción del modelo de IA (Fiabilidad del componente de IA): umbral &gt;=80% exactitud y &gt;=75% sensibilidad en el conjunto de validación antes de habilitarse en producción</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Administrador, Técnico, Trabajador agrícola</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Sin evidencia</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>RNF-16</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>RNF</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>CU-06</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>N/A (RNF, sin HU individual)</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>N/A (RNF, sin HU individual)</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>AIIntegrationModule</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>N/A (no visual)</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>CP-RNF-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Especificación del equipo</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Explicabilidad de las recomendaciones de IA (Transparencia): 100% de las alertas deben mostrar al menos un factor explicativo</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Administrador, Técnico, Trabajador agrícola</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Sin evidencia</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>RNF-17</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>RNF</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>CU-06</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>N/A (RNF, sin HU individual)</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>N/A (RNF, sin HU individual)</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>AIIntegrationModule</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>MU-06</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>CP-RNF-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Especificación del equipo</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Equidad de desempeño entre cultivos (Equidad): diferencia &lt;=10 puntos porcentuales en la tasa de falsos negativos entre cacao y plátano</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Administrador, Técnico, Trabajador agrícola</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Sin evidencia</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>RNF-18</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>RNF</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>CU-06</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>N/A (RNF, sin HU individual)</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>N/A (RNF, sin HU individual)</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>AIIntegrationModule</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>N/A (no visual)</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>CP-RNF-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Especificación del equipo</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Supervisión humana obligatoria antes de cualquier acción automática (Supervisión humana): 0 acciones automáticas sobre datos del sistema sin confirmación humana</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Administrador, Técnico, Trabajador agrícola</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Sin evidencia</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>RNF-19</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>RNF</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>CU-06</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>N/A (RNF, sin HU individual)</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>N/A (RNF, sin HU individual)</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>AIIntegrationModule</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>MU-06</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>CP-RNF-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Especificación del equipo</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Monitoreo continuo del desempeño del modelo en producción (Monitoreo): &gt;=90% de alertas con retroalimentación registrada dentro de 7 días</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Administrador, Técnico, Trabajador agrícola</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Sin evidencia</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>RNF-20</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>RNF</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>CU-06</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>N/A (RNF, sin HU individual)</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>N/A (RNF, sin HU individual)</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>AIIntegrationModule</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>N/A (no visual)</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>CP-RNF-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Especificación del equipo</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Clasificación de riesgo de las recomendaciones de IA (Gestión de riesgo): 100% de los tipos de alerta con nivel de riesgo asignado y visible en la interfaz</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Administrador, Técnico, Trabajador agrícola</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Sin evidencia</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>RNF-21</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>RNF</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>CU-06</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>N/A (RNF, sin HU individual)</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>N/A (RNF, sin HU individual)</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>AIIntegrationModule</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>MU-06</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>CP-RNF-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>